<commit_message>
update excel file and some handle
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
@@ -1,32 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SES_GROUP\12-05-2022 FILE MAU EXCEL\MẪU CÓ SỐ LÔ VÀ HẠN SỬ DỤNG\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5D42463-2D9C-4A33-AB17-B84DD5731EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1AF43CFE-FB0D-429C-9C56-4134A49B1F97}"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -34,18 +28,17 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>ASIA</author>
   </authors>
   <commentList>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{27CB0DBE-9DF0-43A7-B197-5835C8BD2711}">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
@@ -58,22 +51,20 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{EEB5EE67-509D-4CAC-9171-CC635056113A}">
+    <comment ref="N1" authorId="0">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t>Số lô</t>
         </r>
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
             <charset val="1"/>
           </rPr>
@@ -81,63 +72,58 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{5FD23B0F-DE17-469D-855E-69FF88064F64}">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t>Hạn sử dụng</t>
         </r>
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0" xr:uid="{E5DE7EF0-1789-472A-B990-086017A5115D}">
+    <comment ref="S1" authorId="0">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t>Ghi chú</t>
         </r>
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t>:
 ThanhTien = SoLuong x DonGia</t>
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0" xr:uid="{2B216CF0-1708-4D41-AF64-DC21F59C32E0}">
+    <comment ref="U1" authorId="0">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t xml:space="preserve">Ghi chú:
 </t>
@@ -145,9 +131,8 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t>TienThue: Tiền thuế của mỗi sản phẩm</t>
         </r>
@@ -155,9 +140,8 @@
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t>. 
 Tiền thuế = (ThanhTien x ThueSuat)/ 100</t>
@@ -165,33 +149,30 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0" xr:uid="{15B2EC50-FD26-4FC2-BC2D-FA419287C838}">
+    <comment ref="V1" authorId="0">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t>Tính chất hàng hóa, dịch vụ</t>
         </r>
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <family val="2"/>
+            <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
 1: HH/DV
@@ -206,7 +187,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="58">
+  <si>
+    <t>MaHD(*)</t>
+  </si>
   <si>
     <t>MaSoThue</t>
   </si>
@@ -244,6 +228,12 @@
     <t>MaHangHoa</t>
   </si>
   <si>
+    <t>SoLo</t>
+  </si>
+  <si>
+    <t>HanSuDung</t>
+  </si>
+  <si>
     <t>DonViTinh</t>
   </si>
   <si>
@@ -277,57 +267,57 @@
     <t>CÔNG TY A</t>
   </si>
   <si>
+    <t>Địa chỉ A</t>
+  </si>
+  <si>
     <t>xxx@gmail.com</t>
   </si>
   <si>
+    <t>VND</t>
+  </si>
+  <si>
+    <t>Sản phẩm 01</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>23/06/2022</t>
+  </si>
+  <si>
+    <t>Chuyến</t>
+  </si>
+  <si>
+    <t>Sản phẩm 02</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>Kg</t>
+  </si>
+  <si>
+    <t>Sản phẩm 03</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>M3</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
-    <t>VND</t>
-  </si>
-  <si>
-    <t>Sản phẩm 01</t>
-  </si>
-  <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>Chuyến</t>
-  </si>
-  <si>
-    <t>Sản phẩm 02</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>Kg</t>
-  </si>
-  <si>
-    <t>Sản phẩm 03</t>
-  </si>
-  <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t>M3</t>
+    <t>Gói hàng 01</t>
+  </si>
+  <si>
+    <t>ABC</t>
   </si>
   <si>
     <t>3</t>
   </si>
   <si>
-    <t>Gói hàng 01</t>
-  </si>
-  <si>
-    <t>ABC</t>
-  </si>
-  <si>
-    <t>Địa chỉ A</t>
-  </si>
-  <si>
-    <t>MaHD(*)</t>
-  </si>
-  <si>
     <t>Sản phẩm A</t>
   </si>
   <si>
@@ -337,58 +327,58 @@
     <t>Sản phẩm C</t>
   </si>
   <si>
+    <t>END</t>
+  </si>
+  <si>
     <t>Hình thức thanh toán</t>
   </si>
   <si>
+    <t>Tính chất hàng hóa, dịch vụ</t>
+  </si>
+  <si>
     <t>1: Tiền mặt</t>
   </si>
   <si>
+    <t>1: HH/DV</t>
+  </si>
+  <si>
     <t>2: Chuyển khoản</t>
   </si>
   <si>
+    <t>2: KM</t>
+  </si>
+  <si>
     <t>3: Tiền mặt/ chuyển khoản</t>
   </si>
   <si>
+    <t>3: CK</t>
+  </si>
+  <si>
     <t>4: Đối trừ công nợ</t>
   </si>
   <si>
+    <t>4: Ghi chú</t>
+  </si>
+  <si>
     <t>5: Không thu tiền</t>
-  </si>
-  <si>
-    <t>Tính chất hàng hóa, dịch vụ</t>
-  </si>
-  <si>
-    <t>1: HH/DV</t>
-  </si>
-  <si>
-    <t>2: KM</t>
-  </si>
-  <si>
-    <t>3: CK</t>
-  </si>
-  <si>
-    <t>4: Ghi chú</t>
-  </si>
-  <si>
-    <t>SoLo</t>
-  </si>
-  <si>
-    <t>HanSuDung</t>
-  </si>
-  <si>
-    <t>23/06/2022</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -396,43 +386,184 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <color indexed="81"/>
       <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
-      <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <charset val="134"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -447,18 +578,204 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -466,42 +783,328 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -550,7 +1153,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -583,26 +1186,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -635,23 +1221,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -793,152 +1362,147 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ADB66B4-B301-41ED-B48F-710FCDC6CB0D}">
-  <dimension ref="A1:W8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:W9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.8571428571429" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="6" width="19.140625" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="12.7142857142857" customWidth="1"/>
+    <col min="5" max="6" width="19.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="15.2857142857143" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="22.140625" style="7" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" customWidth="1"/>
+    <col min="9" max="9" width="12.8571428571429" customWidth="1"/>
+    <col min="10" max="10" width="22.1428571428571" style="2" customWidth="1"/>
+    <col min="11" max="11" width="11.5714285714286" customWidth="1"/>
+    <col min="12" max="12" width="15.4285714285714" customWidth="1"/>
     <col min="13" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="13.85546875" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="4"/>
-    <col min="18" max="18" width="9.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.8571428571429" customWidth="1"/>
+    <col min="17" max="17" width="9.14285714285714" style="3"/>
+    <col min="18" max="18" width="9.57142857142857" style="4" customWidth="1"/>
     <col min="19" max="19" width="13" customWidth="1"/>
-    <col min="20" max="20" width="12.140625" customWidth="1"/>
-    <col min="21" max="21" width="11.85546875" customWidth="1"/>
+    <col min="20" max="20" width="12.1428571428571" customWidth="1"/>
+    <col min="21" max="21" width="11.8571428571429" customWidth="1"/>
     <col min="22" max="22" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>39</v>
+    <row r="1" spans="1:23">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="2">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" t="s">
-        <v>54</v>
-      </c>
-      <c r="O1" t="s">
-        <v>55</v>
-      </c>
-      <c r="P1" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" s="7">
-        <v>2</v>
-      </c>
       <c r="K2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N2">
         <v>1</v>
       </c>
       <c r="O2" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="P2" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q2" s="4">
+        <v>32</v>
+      </c>
+      <c r="Q2" s="3">
         <v>1</v>
       </c>
-      <c r="R2" s="5">
+      <c r="R2" s="4">
         <v>480000</v>
       </c>
       <c r="S2">
@@ -957,29 +1521,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="L3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="M3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="N3">
         <v>2</v>
       </c>
       <c r="O3" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="P3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q3" s="4">
+        <v>35</v>
+      </c>
+      <c r="Q3" s="3">
         <v>2</v>
       </c>
-      <c r="R3" s="5">
+      <c r="R3" s="4">
         <v>1600</v>
       </c>
       <c r="S3">
@@ -998,29 +1562,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="L4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="M4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="N4">
         <v>2</v>
       </c>
       <c r="O4" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="P4" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q4" s="4">
+        <v>38</v>
+      </c>
+      <c r="Q4" s="3">
         <v>3</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="4">
         <v>480000</v>
       </c>
       <c r="S4">
@@ -1039,26 +1603,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23">
       <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" s="7">
+        <v>39</v>
+      </c>
+      <c r="J5" s="2">
         <v>2</v>
       </c>
       <c r="K5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="M5" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q5" s="4">
+        <v>41</v>
+      </c>
+      <c r="Q5" s="3">
         <v>3</v>
       </c>
-      <c r="R5" s="5">
+      <c r="R5" s="4">
         <v>230000</v>
       </c>
       <c r="S5">
@@ -1079,23 +1643,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23">
       <c r="A6" t="s">
-        <v>35</v>
-      </c>
-      <c r="J6" s="7">
+        <v>42</v>
+      </c>
+      <c r="J6" s="2">
         <v>2</v>
       </c>
       <c r="K6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L6" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q6" s="4">
+        <v>43</v>
+      </c>
+      <c r="Q6" s="3">
         <v>1</v>
       </c>
-      <c r="R6" s="5">
+      <c r="R6" s="4">
         <v>200000</v>
       </c>
       <c r="S6">
@@ -1116,17 +1680,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="L7" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q7" s="4">
+        <v>44</v>
+      </c>
+      <c r="Q7" s="3">
         <v>2</v>
       </c>
-      <c r="R7" s="5">
+      <c r="R7" s="4">
         <v>2900000</v>
       </c>
       <c r="S7">
@@ -1147,17 +1711,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="L8" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q8" s="4">
+        <v>45</v>
+      </c>
+      <c r="Q8" s="3">
         <v>3</v>
       </c>
-      <c r="R8" s="5">
+      <c r="R8" s="4">
         <v>2300000</v>
       </c>
       <c r="S8">
@@ -1178,70 +1742,77 @@
         <v>1</v>
       </c>
     </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6825431-CD75-4952-89A8-789BAD2B1937}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="32.5703125" customWidth="1"/>
-    <col min="2" max="2" width="25.5703125" customWidth="1"/>
+    <col min="1" max="1" width="32.5714285714286" customWidth="1"/>
+    <col min="2" max="2" width="25.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B1" s="8" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>44</v>
       </c>
       <c r="B2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add the ma so ĐVQHNS on invoice crud
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
@@ -30,10 +30,23 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
+    <author>trann</author>
     <author>ASIA</author>
   </authors>
   <commentList>
-    <comment ref="J1" authorId="0">
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Mã số đơn vị có quan hệ với ngân sách (chỉ tồn tại ký tự số)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -51,7 +64,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="O1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -72,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0">
+    <comment ref="P1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -94,7 +107,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0">
+    <comment ref="T1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -116,7 +129,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0">
+    <comment ref="V1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -157,7 +170,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0">
+    <comment ref="W1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -187,7 +200,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="59">
   <si>
     <t>MaHD(*)</t>
   </si>
@@ -201,6 +214,9 @@
     <t>TenDonVi</t>
   </si>
   <si>
+    <t>Mã số ĐVQHNS</t>
+  </si>
+  <si>
     <t>DiaChiKhachHang</t>
   </si>
   <si>
@@ -261,7 +277,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>0107521365</t>
+    <t>xxxxx</t>
   </si>
   <si>
     <t>CÔNG TY A</t>
@@ -390,13 +406,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -539,11 +548,6 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -552,6 +556,11 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
@@ -560,10 +569,15 @@
     <font>
       <sz val="9"/>
       <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -650,19 +664,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -884,97 +886,103 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -983,10 +991,10 @@
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -995,10 +1003,10 @@
     <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1007,10 +1015,10 @@
     <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1019,13 +1027,7 @@
     <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1368,30 +1370,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:W9"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11.8571428571429" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="12.7142857142857" customWidth="1"/>
-    <col min="5" max="6" width="19.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="15.2857142857143" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="12.8571428571429" customWidth="1"/>
-    <col min="10" max="10" width="22.1428571428571" style="2" customWidth="1"/>
-    <col min="11" max="11" width="11.5714285714286" customWidth="1"/>
-    <col min="12" max="12" width="15.4285714285714" customWidth="1"/>
-    <col min="13" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="13.8571428571429" customWidth="1"/>
-    <col min="17" max="17" width="9.14285714285714" style="3"/>
-    <col min="18" max="18" width="9.57142857142857" style="4" customWidth="1"/>
-    <col min="19" max="19" width="13" customWidth="1"/>
-    <col min="20" max="20" width="12.1428571428571" customWidth="1"/>
-    <col min="21" max="21" width="11.8571428571429" customWidth="1"/>
-    <col min="22" max="22" width="10" customWidth="1"/>
+    <col min="5" max="5" width="15.4285714285714" customWidth="1"/>
+    <col min="6" max="7" width="19.1428571428571" customWidth="1"/>
+    <col min="8" max="8" width="15.2857142857143" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="12.8571428571429" customWidth="1"/>
+    <col min="11" max="11" width="22.1428571428571" style="2" customWidth="1"/>
+    <col min="12" max="12" width="11.5714285714286" customWidth="1"/>
+    <col min="13" max="13" width="15.4285714285714" customWidth="1"/>
+    <col min="14" max="16" width="14" customWidth="1"/>
+    <col min="17" max="17" width="13.8571428571429" customWidth="1"/>
+    <col min="18" max="18" width="9.14285714285714" style="3"/>
+    <col min="19" max="19" width="9.57142857142857" style="4" customWidth="1"/>
+    <col min="20" max="20" width="13" customWidth="1"/>
+    <col min="21" max="21" width="12.1428571428571" customWidth="1"/>
+    <col min="22" max="22" width="11.8571428571429" customWidth="1"/>
+    <col min="23" max="23" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:24">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1419,16 +1422,16 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
       <c r="N1" t="s">
@@ -1440,13 +1443,13 @@
       <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="S1" s="4" t="s">
         <v>18</v>
       </c>
       <c r="T1" s="8" t="s">
@@ -1461,28 +1464,28 @@
       <c r="W1" s="8" t="s">
         <v>22</v>
       </c>
+      <c r="X1" s="8" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="2" spans="1:23">
+    <row r="2" spans="1:24">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" t="s">
         <v>26</v>
       </c>
       <c r="F2" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="2">
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" s="2">
         <v>2</v>
-      </c>
-      <c r="K2" t="s">
-        <v>28</v>
       </c>
       <c r="L2" t="s">
         <v>29</v>
@@ -1490,261 +1493,264 @@
       <c r="M2" t="s">
         <v>30</v>
       </c>
-      <c r="N2">
+      <c r="N2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2">
         <v>1</v>
-      </c>
-      <c r="O2" t="s">
-        <v>31</v>
       </c>
       <c r="P2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="Q2" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="3">
         <v>1</v>
       </c>
-      <c r="R2" s="4">
+      <c r="S2" s="4">
         <v>480000</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>480000</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>10</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>48000</v>
-      </c>
-      <c r="V2">
-        <v>1</v>
       </c>
       <c r="W2">
         <v>1</v>
       </c>
+      <c r="X2">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:24">
       <c r="A3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="M3" t="s">
         <v>34</v>
       </c>
-      <c r="N3">
+      <c r="N3" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3">
         <v>2</v>
       </c>
-      <c r="O3" t="s">
-        <v>31</v>
-      </c>
       <c r="P3" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q3" s="3">
+        <v>32</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" s="3">
         <v>2</v>
       </c>
-      <c r="R3" s="4">
+      <c r="S3" s="4">
         <v>1600</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>2264000</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>10</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>22640000</v>
-      </c>
-      <c r="V3">
-        <v>1</v>
       </c>
       <c r="W3">
         <v>1</v>
       </c>
+      <c r="X3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:23">
+    <row r="4" spans="1:24">
       <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="L4" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="M4" t="s">
         <v>37</v>
       </c>
-      <c r="N4">
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4">
         <v>2</v>
       </c>
-      <c r="O4" t="s">
-        <v>31</v>
-      </c>
       <c r="P4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q4" s="3">
+        <v>32</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>39</v>
+      </c>
+      <c r="R4" s="3">
         <v>3</v>
       </c>
-      <c r="R4" s="4">
+      <c r="S4" s="4">
         <v>480000</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>1797600</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>10</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>17976000</v>
-      </c>
-      <c r="V4">
-        <v>1</v>
       </c>
       <c r="W4">
         <v>1</v>
       </c>
+      <c r="X4">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="1:23">
+    <row r="5" spans="1:24">
       <c r="A5" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" s="2">
+        <v>40</v>
+      </c>
+      <c r="K5" s="2">
         <v>2</v>
       </c>
-      <c r="K5" t="s">
-        <v>28</v>
-      </c>
       <c r="L5" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="M5" t="s">
         <v>41</v>
       </c>
-      <c r="Q5" s="3">
+      <c r="N5" t="s">
+        <v>42</v>
+      </c>
+      <c r="R5" s="3">
         <v>3</v>
       </c>
-      <c r="R5" s="4">
+      <c r="S5" s="4">
         <v>230000</v>
       </c>
-      <c r="S5">
-        <f>Q5*R5</f>
+      <c r="T5">
+        <f>R5*S5</f>
         <v>690000</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>10</v>
       </c>
-      <c r="U5">
-        <f>(S5*T5)/100</f>
+      <c r="V5">
+        <f>(T5*U5)/100</f>
         <v>69000</v>
-      </c>
-      <c r="V5">
-        <v>1</v>
       </c>
       <c r="W5">
         <v>1</v>
       </c>
+      <c r="X5">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="1:23">
+    <row r="6" spans="1:24">
       <c r="A6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J6" s="2">
+        <v>43</v>
+      </c>
+      <c r="K6" s="2">
         <v>2</v>
       </c>
-      <c r="K6" t="s">
-        <v>28</v>
-      </c>
       <c r="L6" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q6" s="3">
+        <v>29</v>
+      </c>
+      <c r="M6" t="s">
+        <v>44</v>
+      </c>
+      <c r="R6" s="3">
         <v>1</v>
       </c>
-      <c r="R6" s="4">
+      <c r="S6" s="4">
         <v>200000</v>
       </c>
-      <c r="S6">
-        <f t="shared" ref="S6:S8" si="0">Q6*R6</f>
+      <c r="T6">
+        <f t="shared" ref="T6:T8" si="0">R6*S6</f>
         <v>200000</v>
       </c>
-      <c r="T6">
+      <c r="U6">
         <v>8</v>
       </c>
-      <c r="U6">
-        <f t="shared" ref="U6:U8" si="1">(S6*T6)/100</f>
+      <c r="V6">
+        <f t="shared" ref="V6:V8" si="1">(T6*U6)/100</f>
         <v>16000</v>
-      </c>
-      <c r="V6">
-        <v>1</v>
       </c>
       <c r="W6">
         <v>1</v>
       </c>
+      <c r="X6">
+        <v>1</v>
+      </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:24">
       <c r="A7" t="s">
-        <v>42</v>
-      </c>
-      <c r="L7" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q7" s="3">
+        <v>43</v>
+      </c>
+      <c r="M7" t="s">
+        <v>45</v>
+      </c>
+      <c r="R7" s="3">
         <v>2</v>
       </c>
-      <c r="R7" s="4">
+      <c r="S7" s="4">
         <v>2900000</v>
       </c>
-      <c r="S7">
+      <c r="T7">
         <f t="shared" si="0"/>
         <v>5800000</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>10</v>
       </c>
-      <c r="U7">
+      <c r="V7">
         <f t="shared" si="1"/>
         <v>580000</v>
       </c>
-      <c r="V7">
-        <v>1</v>
-      </c>
       <c r="W7">
         <v>1</v>
       </c>
+      <c r="X7">
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:24">
       <c r="A8" t="s">
-        <v>42</v>
-      </c>
-      <c r="L8" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q8" s="3">
+        <v>43</v>
+      </c>
+      <c r="M8" t="s">
+        <v>46</v>
+      </c>
+      <c r="R8" s="3">
         <v>3</v>
       </c>
-      <c r="R8" s="4">
+      <c r="S8" s="4">
         <v>2300000</v>
       </c>
-      <c r="S8">
+      <c r="T8">
         <f t="shared" si="0"/>
         <v>6900000</v>
       </c>
-      <c r="T8">
+      <c r="U8">
         <v>8</v>
       </c>
-      <c r="U8">
+      <c r="V8">
         <f t="shared" si="1"/>
         <v>552000</v>
       </c>
-      <c r="V8">
+      <c r="W8">
         <v>1</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1767,47 +1773,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add cccd and shchieu fields on crud and import vat invoice
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="23040" windowHeight="8940"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="1">
+    <comment ref="M1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -64,7 +64,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="1">
+    <comment ref="Q1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -85,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="1">
+    <comment ref="R1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -107,7 +107,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="1">
+    <comment ref="V1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -129,7 +129,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="1">
+    <comment ref="X1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -170,7 +170,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="1">
+    <comment ref="Y1" authorId="1">
       <text>
         <r>
           <rPr>
@@ -200,7 +200,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="61">
   <si>
     <t>MaHD(*)</t>
   </si>
@@ -214,7 +214,7 @@
     <t>TenDonVi</t>
   </si>
   <si>
-    <t>Mã số ĐVQHNS</t>
+    <t>MaSoĐVQHNS</t>
   </si>
   <si>
     <t>DiaChiKhachHang</t>
@@ -224,6 +224,12 @@
   </si>
   <si>
     <t>SoDienThoaiKH</t>
+  </si>
+  <si>
+    <t>SoCCCD</t>
+  </si>
+  <si>
+    <t>SoHoChieu</t>
   </si>
   <si>
     <t>SoTaiKhoan</t>
@@ -550,6 +556,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
@@ -557,21 +573,11 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
+      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
@@ -1031,9 +1037,10 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1370,7 +1377,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:Z9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11.8571428571429" customWidth="1"/>
@@ -1378,24 +1385,24 @@
     <col min="4" max="4" width="12.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="15.4285714285714" customWidth="1"/>
     <col min="6" max="7" width="19.1428571428571" customWidth="1"/>
-    <col min="8" max="8" width="15.2857142857143" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="12.8571428571429" customWidth="1"/>
-    <col min="11" max="11" width="22.1428571428571" style="2" customWidth="1"/>
-    <col min="12" max="12" width="11.5714285714286" customWidth="1"/>
-    <col min="13" max="13" width="15.4285714285714" customWidth="1"/>
-    <col min="14" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="13.8571428571429" customWidth="1"/>
-    <col min="18" max="18" width="9.14285714285714" style="3"/>
-    <col min="19" max="19" width="9.57142857142857" style="4" customWidth="1"/>
-    <col min="20" max="20" width="13" customWidth="1"/>
-    <col min="21" max="21" width="12.1428571428571" customWidth="1"/>
-    <col min="22" max="22" width="11.8571428571429" customWidth="1"/>
-    <col min="23" max="23" width="10" customWidth="1"/>
+    <col min="8" max="10" width="15.2857142857143" style="2" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="12.8571428571429" customWidth="1"/>
+    <col min="13" max="13" width="22.1428571428571" style="3" customWidth="1"/>
+    <col min="14" max="14" width="11.5714285714286" customWidth="1"/>
+    <col min="15" max="15" width="15.4285714285714" customWidth="1"/>
+    <col min="16" max="18" width="14" customWidth="1"/>
+    <col min="19" max="19" width="13.8571428571429" customWidth="1"/>
+    <col min="20" max="20" width="9.14285714285714" style="4"/>
+    <col min="21" max="21" width="9.57142857142857" style="5" customWidth="1"/>
+    <col min="22" max="22" width="13" customWidth="1"/>
+    <col min="23" max="23" width="12.1428571428571" customWidth="1"/>
+    <col min="24" max="24" width="11.8571428571429" customWidth="1"/>
+    <col min="25" max="25" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:26">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1416,28 +1423,28 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="8" t="s">
         <v>14</v>
       </c>
       <c r="P1" t="s">
@@ -1446,311 +1453,317 @@
       <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="U1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="V1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="8" t="s">
+      <c r="W1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="X1" s="9" t="s">
         <v>23</v>
       </c>
+      <c r="Y1" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="9" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:26">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K2" s="2">
+        <v>30</v>
+      </c>
+      <c r="M2" s="3">
         <v>2</v>
-      </c>
-      <c r="L2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M2" t="s">
-        <v>30</v>
       </c>
       <c r="N2" t="s">
         <v>31</v>
       </c>
-      <c r="O2">
+      <c r="O2" t="s">
+        <v>32</v>
+      </c>
+      <c r="P2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q2">
         <v>1</v>
       </c>
-      <c r="P2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>33</v>
-      </c>
-      <c r="R2" s="3">
+      <c r="R2" t="s">
+        <v>34</v>
+      </c>
+      <c r="S2" t="s">
+        <v>35</v>
+      </c>
+      <c r="T2" s="4">
         <v>1</v>
       </c>
-      <c r="S2" s="4">
+      <c r="U2" s="5">
         <v>480000</v>
       </c>
-      <c r="T2">
+      <c r="V2">
         <v>480000</v>
       </c>
-      <c r="U2">
+      <c r="W2">
         <v>10</v>
       </c>
-      <c r="V2">
+      <c r="X2">
         <v>48000</v>
       </c>
-      <c r="W2">
+      <c r="Y2">
         <v>1</v>
       </c>
-      <c r="X2">
+      <c r="Z2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M3" t="s">
+        <v>26</v>
+      </c>
+      <c r="O3" t="s">
+        <v>36</v>
+      </c>
+      <c r="P3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q3">
+        <v>2</v>
+      </c>
+      <c r="R3" t="s">
         <v>34</v>
       </c>
-      <c r="N3" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3">
+      <c r="S3" t="s">
+        <v>38</v>
+      </c>
+      <c r="T3" s="4">
         <v>2</v>
       </c>
-      <c r="P3" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>36</v>
-      </c>
-      <c r="R3" s="3">
+      <c r="U3" s="5">
+        <v>1600</v>
+      </c>
+      <c r="V3">
+        <v>2264000</v>
+      </c>
+      <c r="W3">
+        <v>10</v>
+      </c>
+      <c r="X3">
+        <v>22640000</v>
+      </c>
+      <c r="Y3">
+        <v>1</v>
+      </c>
+      <c r="Z3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O4" t="s">
+        <v>39</v>
+      </c>
+      <c r="P4" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q4">
         <v>2</v>
       </c>
-      <c r="S3" s="4">
-        <v>1600</v>
-      </c>
-      <c r="T3">
-        <v>2264000</v>
-      </c>
-      <c r="U3">
+      <c r="R4" t="s">
+        <v>34</v>
+      </c>
+      <c r="S4" t="s">
+        <v>41</v>
+      </c>
+      <c r="T4" s="4">
+        <v>3</v>
+      </c>
+      <c r="U4" s="5">
+        <v>480000</v>
+      </c>
+      <c r="V4">
+        <v>1797600</v>
+      </c>
+      <c r="W4">
         <v>10</v>
       </c>
-      <c r="V3">
-        <v>22640000</v>
-      </c>
-      <c r="W3">
+      <c r="X4">
+        <v>17976000</v>
+      </c>
+      <c r="Y4">
         <v>1</v>
       </c>
-      <c r="X3">
+      <c r="Z4">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" t="s">
-        <v>37</v>
-      </c>
-      <c r="N4" t="s">
-        <v>38</v>
-      </c>
-      <c r="O4">
+    <row r="5" spans="1:26">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+      <c r="M5" s="3">
         <v>2</v>
       </c>
-      <c r="P4" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>39</v>
-      </c>
-      <c r="R4" s="3">
+      <c r="N5" t="s">
+        <v>31</v>
+      </c>
+      <c r="O5" t="s">
+        <v>43</v>
+      </c>
+      <c r="P5" t="s">
+        <v>44</v>
+      </c>
+      <c r="T5" s="4">
         <v>3</v>
       </c>
-      <c r="S4" s="4">
-        <v>480000</v>
-      </c>
-      <c r="T4">
-        <v>1797600</v>
-      </c>
-      <c r="U4">
+      <c r="U5" s="5">
+        <v>230000</v>
+      </c>
+      <c r="V5">
+        <f>T5*U5</f>
+        <v>690000</v>
+      </c>
+      <c r="W5">
         <v>10</v>
       </c>
-      <c r="V4">
-        <v>17976000</v>
-      </c>
-      <c r="W4">
+      <c r="X5">
+        <f>(V5*W5)/100</f>
+        <v>69000</v>
+      </c>
+      <c r="Y5">
         <v>1</v>
       </c>
-      <c r="X4">
+      <c r="Z5">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
-      <c r="A5" t="s">
-        <v>40</v>
-      </c>
-      <c r="K5" s="2">
+    <row r="6" spans="1:26">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="M6" s="3">
         <v>2</v>
       </c>
-      <c r="L5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M5" t="s">
-        <v>41</v>
-      </c>
-      <c r="N5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R5" s="3">
-        <v>3</v>
-      </c>
-      <c r="S5" s="4">
-        <v>230000</v>
-      </c>
-      <c r="T5">
-        <f>R5*S5</f>
-        <v>690000</v>
-      </c>
-      <c r="U5">
-        <v>10</v>
-      </c>
-      <c r="V5">
-        <f>(T5*U5)/100</f>
-        <v>69000</v>
-      </c>
-      <c r="W5">
+      <c r="N6" t="s">
+        <v>31</v>
+      </c>
+      <c r="O6" t="s">
+        <v>46</v>
+      </c>
+      <c r="T6" s="4">
         <v>1</v>
       </c>
-      <c r="X5">
+      <c r="U6" s="5">
+        <v>200000</v>
+      </c>
+      <c r="V6">
+        <f t="shared" ref="V6:V8" si="0">T6*U6</f>
+        <v>200000</v>
+      </c>
+      <c r="W6">
+        <v>8</v>
+      </c>
+      <c r="X6">
+        <f t="shared" ref="X6:X8" si="1">(V6*W6)/100</f>
+        <v>16000</v>
+      </c>
+      <c r="Y6">
         <v>1</v>
       </c>
+      <c r="Z6">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="1:24">
-      <c r="A6" t="s">
-        <v>43</v>
-      </c>
-      <c r="K6" s="2">
+    <row r="7" spans="1:26">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="O7" t="s">
+        <v>47</v>
+      </c>
+      <c r="T7" s="4">
         <v>2</v>
       </c>
-      <c r="L6" t="s">
-        <v>29</v>
-      </c>
-      <c r="M6" t="s">
-        <v>44</v>
-      </c>
-      <c r="R6" s="3">
-        <v>1</v>
-      </c>
-      <c r="S6" s="4">
-        <v>200000</v>
-      </c>
-      <c r="T6">
-        <f t="shared" ref="T6:T8" si="0">R6*S6</f>
-        <v>200000</v>
-      </c>
-      <c r="U6">
-        <v>8</v>
-      </c>
-      <c r="V6">
-        <f t="shared" ref="V6:V8" si="1">(T6*U6)/100</f>
-        <v>16000</v>
-      </c>
-      <c r="W6">
-        <v>1</v>
-      </c>
-      <c r="X6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24">
-      <c r="A7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M7" t="s">
-        <v>45</v>
-      </c>
-      <c r="R7" s="3">
-        <v>2</v>
-      </c>
-      <c r="S7" s="4">
+      <c r="U7" s="5">
         <v>2900000</v>
       </c>
-      <c r="T7">
+      <c r="V7">
         <f t="shared" si="0"/>
         <v>5800000</v>
       </c>
-      <c r="U7">
+      <c r="W7">
         <v>10</v>
       </c>
-      <c r="V7">
+      <c r="X7">
         <f t="shared" si="1"/>
         <v>580000</v>
       </c>
-      <c r="W7">
+      <c r="Y7">
         <v>1</v>
       </c>
-      <c r="X7">
+      <c r="Z7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>43</v>
-      </c>
-      <c r="M8" t="s">
-        <v>46</v>
-      </c>
-      <c r="R8" s="3">
+        <v>45</v>
+      </c>
+      <c r="O8" t="s">
+        <v>48</v>
+      </c>
+      <c r="T8" s="4">
         <v>3</v>
       </c>
-      <c r="S8" s="4">
+      <c r="U8" s="5">
         <v>2300000</v>
       </c>
-      <c r="T8">
+      <c r="V8">
         <f t="shared" si="0"/>
         <v>6900000</v>
       </c>
-      <c r="U8">
+      <c r="W8">
         <v>8</v>
       </c>
-      <c r="V8">
+      <c r="X8">
         <f t="shared" si="1"/>
         <v>552000</v>
       </c>
-      <c r="W8">
+      <c r="Y8">
         <v>1</v>
       </c>
-      <c r="X8">
+      <c r="Z8">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1773,47 +1786,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add feature of product (hanghoadactrung) when import vat invoice
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8940"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -191,7 +191,315 @@
 1: HH/DV
 2: KM
 3: CK
-4: Ghi chú</t>
+4: Ghi chú
+5: Hàng hóa đặc trưng</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">Loại hàng hóa đặc trưng áp dụng khi Tính chất là 5:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>1</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">: Hàng hóa là xe ô tô, xe mô tô 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>2</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">: Dịch vụ vận chuyển
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>3</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">: Dịch vụ vận chuyển trên nền tảng số, TMĐT
+Trong trường hợp Tính chất không phải là </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>5</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>, bỏ trống</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">Số khung áp dụng khi Loại hàng hóa đặc trưng là 1:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">Nếu Loại hàng hóa đặc trưng khác </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>1</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>, bỏ trống</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">Số máy áp dụng khi Loại hàng hóa đặc trưng là 1:
+Nếu Loại hàng hóa đặc trưng khác 1, bỏ trống
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Biển kiểm soát phương tiện vận chuyển áp dụng khi Loại hàng hóa đặc trưng là 2:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Nếu Loại hàng hóa đặc trưng khác </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>2</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">, bỏ trống
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Tên người gửi hàng áp dụng khi Loại hàng hóa đặc trưng là 3:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Nếu Loại hàng hóa đặc trưng khác </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>3</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>, bỏ trống</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Địa chỉ người gửi hàng áp dụng khi Loại hàng hóa đặc trưng là 3:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Nếu Loại hàng hóa đặc trưng khác </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>3</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">, bỏ trống
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Số định danh người gửi hàng áp dụng khi Loại hàng hóa đặc trưng là 3:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Nếu Loại hàng hóa đặc trưng khác </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>3</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">, bỏ trống
+</t>
         </r>
       </text>
     </comment>
@@ -200,7 +508,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="69">
   <si>
     <t>MaHD(*)</t>
   </si>
@@ -278,6 +586,30 @@
   </si>
   <si>
     <t>TyGia(*)</t>
+  </si>
+  <si>
+    <t>LoaiHangHoaDacTrung</t>
+  </si>
+  <si>
+    <t>SoKhung</t>
+  </si>
+  <si>
+    <t>SoMay</t>
+  </si>
+  <si>
+    <t>BienKiemSoatPTVC</t>
+  </si>
+  <si>
+    <t>TenNguoiGuiHang</t>
+  </si>
+  <si>
+    <t>DiaChiNguoiGuiHang</t>
+  </si>
+  <si>
+    <t>MSTNguoiGuiHang</t>
+  </si>
+  <si>
+    <t>SoDinhDanhNguoiGuiHang</t>
   </si>
   <si>
     <t>1</t>
@@ -395,7 +727,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -556,14 +888,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
     </font>
     <font>
       <b/>
@@ -572,18 +910,18 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Tahoma"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Tahoma"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -605,6 +943,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -913,7 +1257,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -937,16 +1281,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -955,89 +1299,89 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1058,6 +1402,7 @@
     <xf numFmtId="1" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1377,7 +1722,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:AH10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11.8571428571429" customWidth="1"/>
@@ -1399,9 +1744,18 @@
     <col min="23" max="23" width="12.1428571428571" customWidth="1"/>
     <col min="24" max="24" width="11.8571428571429" customWidth="1"/>
     <col min="25" max="25" width="10" customWidth="1"/>
+    <col min="26" max="26" width="9" customWidth="1"/>
+    <col min="27" max="27" width="22.5714285714286" style="2" customWidth="1"/>
+    <col min="28" max="28" width="19" style="2" customWidth="1"/>
+    <col min="29" max="29" width="14.1428571428571" style="2" customWidth="1"/>
+    <col min="30" max="30" width="19.5714285714286" style="2" customWidth="1"/>
+    <col min="31" max="31" width="19" style="2" customWidth="1"/>
+    <col min="32" max="32" width="21.2857142857143" style="2" customWidth="1"/>
+    <col min="33" max="33" width="19" style="2" customWidth="1"/>
+    <col min="34" max="34" width="27" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:34">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1479,44 +1833,68 @@
       </c>
       <c r="Z1" s="9" t="s">
         <v>25</v>
+      </c>
+      <c r="AA1" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:26">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="M2" s="3">
         <v>2</v>
       </c>
       <c r="N2" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="O2" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="P2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="Q2">
         <v>1</v>
       </c>
       <c r="R2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="S2" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="T2" s="4">
         <v>1</v>
@@ -1542,22 +1920,22 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="O3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="P3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="Q3">
         <v>2</v>
       </c>
       <c r="R3" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="S3" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="T3" s="4">
         <v>2</v>
@@ -1583,22 +1961,22 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="O4" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="P4" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="Q4">
         <v>2</v>
       </c>
       <c r="R4" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="S4" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="T4" s="4">
         <v>3</v>
@@ -1624,19 +2002,19 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="M5" s="3">
         <v>2</v>
       </c>
       <c r="N5" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="O5" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="P5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="T5" s="4">
         <v>3</v>
@@ -1664,16 +2042,16 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="M6" s="3">
         <v>2</v>
       </c>
       <c r="N6" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="O6" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="T6" s="4">
         <v>1</v>
@@ -1701,10 +2079,10 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="O7" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="T7" s="4">
         <v>2</v>
@@ -1732,10 +2110,10 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="O8" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="T8" s="4">
         <v>3</v>
@@ -1763,8 +2141,16 @@
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>49</v>
-      </c>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="8:21">
+      <c r="H10"/>
+      <c r="I10"/>
+      <c r="J10"/>
+      <c r="M10"/>
+      <c r="T10"/>
+      <c r="U10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1786,47 +2172,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: rollback new method payment is empty on invoices
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/einvoices/MauUploadHD01-TT78.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11460"/>
+    <workbookView windowWidth="28800" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -60,8 +60,7 @@
 2: Chuyển khoản
 3: Tiền mặt/ chuyển khoản
 4: Đối trừ công nợ
-5: Không thu tiền
-6: “” (Không ghi hình thức)</t>
+5: Không thu tiền</t>
         </r>
       </text>
     </comment>
@@ -890,13 +889,14 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
     </font>
     <font>
       <b/>
@@ -912,14 +912,13 @@
     <font>
       <b/>
       <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <name val="Times New Roman"/>
-      <charset val="0"/>
     </font>
   </fonts>
   <fills count="35">

</xml_diff>